<commit_message>
Update M4_Notes in v8 workbook to reflect closed M4-M2 loop and current results
</commit_message>
<xml_diff>
--- a/models/SPUR_Combined_Model_v8.xlsx
+++ b/models/SPUR_Combined_Model_v8.xlsx
@@ -1966,7 +1966,7 @@
     <t>§3 FINDING: Model 2's $60/MWh BTM price is below LCOE for solar and wind</t>
   </si>
   <si>
-    <t>Base-case co-location LCOE net of tax equity: Solar $79.70, Wind $69.89, Geothermal $55.05. Model 2 v7 uses a flat $60 BTM input for all three. At $60, solar is selling ~$20 below cost and wind ~$10 below cost at 8% WACC; only geothermal clears its floor. This is consistent with Model 2's own unlevered IRRs (solar 1.3%, wind 2.6%, geo 5.0% co-loc: all below 8%) and with the earlier finding that solar cannot be rescued by co-location. The $60 figure came from the 'industry 10–20% discount to energy PPA' convention, which is benchmarked to the $72 energy-only PPA and is blind to the developer's cost.</t>
+    <t xml:space="preserve">Base-case co-location LCOE net of tax equity: Solar $79.70, Wind $69.89, Geothermal $55.05. At the industry-convention flat $60 BTM price (Inputs!B27 = 1), solar sells ~$20 below cost and wind ~$10 below cost at 8% WACC; only geothermal clears its floor. Consistent with this, at a flat $60 co-location lowers developer levered IRR relative to the deferred-construction baseline for every configuration, ITC case and delay tested (Results rows 24–55; e.g. 4-yr delay, 30% ITC: solar 4.4% vs 12.6%, wind 10.1% vs 18.9%, geothermal 18.8% vs 25.1%). The $60 figure comes from the 'industry 10–20% discount to energy PPA' convention, which is benchmarked to the $72 energy-only PPA and is blind to the developer's cost.</t>
   </si>
   <si>
     <t>§4 FINDING: the true negotiation zone is much wider than the framework expected, because the ceiling is higher</t>
@@ -1987,16 +1987,16 @@
     <t>P_max is solved from the Model 3 Phase-2 cost equation: P such that DC all-in cost = Ceiling_A × (1 − min_savings). P_min is the LCOE floor. Range width: Solar $74.50, Wind $62.65, Geo $67.16: a deal exists for all three at 20% minimum DC savings and 8% developer WACC. Solar's range is widest because its low coverage ratio (29%) means the BTM price has little weight in the DC's blended cost, so the DC is price-insensitive to it. This is a double-edged result: the DC will accept a high solar BTM price, but the developer earns it on only 29% of the DC's load.</t>
   </si>
   <si>
-    <t xml:space="preserve">§7  What is NOT closed in this iteration</t>
-  </si>
-  <si>
-    <t>(a) The M4→M2 loop is not auto-linked: Model 2 v7 has a single global BTM cell (Inputs!B19). To close the loop, set B19 to each config's selected price in turn and read the levered IRR: or add a per-config BTM row to Model 2. (b) The IRR shown in M4_Pricing SEC 4 is Model 2's live value at $60, not at the selected price; it is a proxy. (c) LCOE uses 8% flat; a config-specific WACC (geothermal lower risk → lower WACC → lower floor) would widen the geothermal zone further. (d) Bargaining share α is a lever, not an estimate: practitioner interviews (Q4 in Chien questions, tax-equity market conditions) are the intended source. (e) Carbon scenarios from M1 are not yet wired into the ceiling; C30/C60 would raise Ceiling_C by $13/$26 and Ceiling_A by roughly the same (higher spot passes through to the sleeved PPA).</t>
+    <t xml:space="preserve">§7  Loop closure status and open items (updated for v8)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">(a) CLOSED in v8: the M4→M2 loop is linked. Configurations row 16 takes each configuration's selected Model 4 price when Inputs!B27 = 2; set B27 = 1 to reproduce the flat $60 runs. (b) CLOSED in v8: the developer IRR in M4_Pricing SEC 4 is Model 2's live levered IRR at the effective (Model 4) BTM price, not a $60 proxy. (c) OPEN: Model 3 Structure C still uses its own BTM placeholder (M3_Inputs!B25 = $62) rather than the selected Model 4 price; M4_Pricing row 27 computes the DC's Phase-2 cost at the selected price directly. (d) OPEN: LCOE uses 8% flat; a config-specific WACC (geothermal lower risk → lower WACC → lower floor) would widen the geothermal zone further. (e) OPEN: Bargaining share α is a lever, not an estimate: practitioner interviews (Q4 in Chien questions, tax-equity market conditions) are the intended source. (f) OPEN: Carbon scenarios from M1 are not yet wired into the ceiling; C30/C60 would raise Ceiling_C by $13/$26 and Ceiling_A by roughly the same (higher spot passes through to the sleeved PPA).</t>
   </si>
   <si>
     <t xml:space="preserve">§8  Implication for H1/H2 restatement</t>
   </si>
   <si>
-    <t>H1 (developer IRR +3–6 pp) was tested in Model 2 at $60 BTM. At Model-4-consistent prices, the co-location uplift is larger for all configs and solar likely crosses the 10% hurdle. H2 (DC saves 20–35%) holds at the midpoint price for all configs in Phase 2 (26–28%). The restated hypothesis should be joint: 'there exists a BTM price at which the developer clears WACC and the DC saves ≥20%, for all three configurations, with the geothermal zone widest on the developer side and the solar zone widest on the DC side.'</t>
+    <t xml:space="preserve">H1 (developer IRR +3–6 pp) was originally tested in Model 2 at a flat $60 BTM price, where co-location lowers IRR for all configurations. At the Model 4 price (α = 0.5), in the base case of a 4-year delay and 30% ITC, co-location changes developer levered IRR by −0.8 pp for solar (11.8% vs 12.6%: it clears the 10% hurdle but not the waiting baseline), +5.5 pp for wind and +8.0 pp for geothermal, and raises developer NPV for all three. From Fig2_Breakeven, co-location beats waiting once the delay exceeds about 4 years for solar and 2 years for wind, and at every delay tested for geothermal. H2 (DC saves 20–35%) holds at the midpoint price for all configs in Phase 2 (26–28%). The restated hypothesis should be joint: 'there exists a BTM price at which the developer clears WACC and the DC saves ≥20%, for all three configurations, with the geothermal zone widest on the developer side and the solar zone widest on the DC side.'</t>
   </si>
   <si>
     <t>Figure 2 data: developer levered IRR vs queue wait (static sweep values; BTM lever 1 = flat $60, 2 = Model 4 price)</t>

</xml_diff>